<commit_message>
Weeklogs and gitignore (#20)
</commit_message>
<xml_diff>
--- a/Documents/AndrewPrestaWeeklyLogs/PrestaAndrewWeeklogs.xlsx
+++ b/Documents/AndrewPrestaWeeklyLogs/PrestaAndrewWeeklogs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Downloads\DeSales\SWE\Documents\AndrewPrestaWeeklyLogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E8D1BB-B912-48E0-B985-64FD45FBF68F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58657684-F074-4737-9654-1CF329F05F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="861" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="861" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="14" r:id="rId1"/>
@@ -22,6 +22,8 @@
     <sheet name="Feb 22-Mar 1" sheetId="21" r:id="rId7"/>
     <sheet name="Mar 1 - Mar 8" sheetId="22" r:id="rId8"/>
     <sheet name="Mar 15 - Mar 22" sheetId="24" r:id="rId9"/>
+    <sheet name="Mar 22 - Mar 29" sheetId="25" r:id="rId10"/>
+    <sheet name="Mar 29 - Apr 12" sheetId="26" r:id="rId11"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="45">
   <si>
     <t>Date on which you worked on the project.</t>
   </si>
@@ -162,6 +164,33 @@
     <t>1. Filled out use case #4 tasks and acceptance criteria.
 2. Assigned a task for use case #2 and #6.
 3. Started implementing the previous IDE and terminal in a clean and structured way.</t>
+  </si>
+  <si>
+    <t>3/23/2026, 3/25/2026, 3/27/2026</t>
+  </si>
+  <si>
+    <t>1. Continued implementing the previous IDE and terminal in a clean and structured way.
+2. Created classes for registering and getting a single socket, and registering input and output.
+3. Created classes for ProcessManager and TerminalManager for handling streaming and writing to terminal respectively.
+4. Created more separation handlers and a test class to run the code.</t>
+  </si>
+  <si>
+    <t>3/30/2026, 4/1/2026, 4/3/2026</t>
+  </si>
+  <si>
+    <t>1, 4, 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1, </t>
+  </si>
+  <si>
+    <t>Use Case #4: Using IDE</t>
+  </si>
+  <si>
+    <t>1. Met with the team to pick tasks and develop the Spring Planning document</t>
+  </si>
+  <si>
+    <t>Sprint Planning, Use Case #4: Using IDE</t>
   </si>
 </sst>
 </file>
@@ -631,12 +660,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD054709-500D-4F76-8B36-C67C0620C98A}">
   <dimension ref="A1:Y8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:25" s="1" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="19" t="s">
         <v>5</v>
       </c>
@@ -683,20 +712,20 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
       <c r="M2" s="4"/>
-      <c r="N2" s="22">
-        <v>46043</v>
-      </c>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
-      <c r="X2" s="6"/>
-      <c r="Y2" s="7"/>
+      <c r="N2" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="24"/>
     </row>
     <row r="3" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
@@ -714,8 +743,8 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="4"/>
-      <c r="N3" s="5">
-        <v>1</v>
+      <c r="N3" s="5" t="s">
+        <v>40</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
@@ -746,7 +775,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="4"/>
       <c r="N4" s="5" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
@@ -776,20 +805,20 @@
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
       <c r="M5" s="10"/>
-      <c r="N5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
-      <c r="T5" s="6"/>
-      <c r="U5" s="6"/>
-      <c r="V5" s="6"/>
-      <c r="W5" s="6"/>
-      <c r="X5" s="6"/>
-      <c r="Y5" s="7"/>
+      <c r="N5" s="5">
+        <v>2.1</v>
+      </c>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+      <c r="Y5" s="12"/>
     </row>
     <row r="6" spans="1:25" ht="162" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
@@ -808,7 +837,7 @@
       <c r="L6" s="14"/>
       <c r="M6" s="15"/>
       <c r="N6" s="16" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
@@ -839,252 +868,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="4"/>
       <c r="N7" s="5">
-        <v>1</v>
-      </c>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
-      <c r="T7" s="6"/>
-      <c r="U7" s="6"/>
-      <c r="V7" s="6"/>
-      <c r="W7" s="6"/>
-      <c r="X7" s="6"/>
-      <c r="Y7" s="7"/>
-    </row>
-    <row r="8" spans="1:25" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A6:M6"/>
-    <mergeCell ref="A7:M7"/>
-    <mergeCell ref="N4:Y4"/>
-    <mergeCell ref="N7:Y7"/>
-    <mergeCell ref="N6:Y6"/>
-    <mergeCell ref="N5:Y5"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="N2:Y2"/>
-    <mergeCell ref="N3:Y3"/>
-    <mergeCell ref="N1:Y1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Y8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:25" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20"/>
-      <c r="T1" s="20"/>
-      <c r="U1" s="20"/>
-      <c r="V1" s="20"/>
-      <c r="W1" s="20"/>
-      <c r="X1" s="20"/>
-      <c r="Y1" s="21"/>
-    </row>
-    <row r="2" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="22">
-        <v>46055</v>
-      </c>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="24"/>
-    </row>
-    <row r="3" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="5">
-        <v>1</v>
-      </c>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="7"/>
-    </row>
-    <row r="4" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
-      <c r="W4" s="6"/>
-      <c r="X4" s="6"/>
-      <c r="Y4" s="7"/>
-    </row>
-    <row r="5" spans="1:25" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-      <c r="W5" s="11"/>
-      <c r="X5" s="11"/>
-      <c r="Y5" s="12"/>
-    </row>
-    <row r="6" spans="1:25" ht="162" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="17"/>
-      <c r="R6" s="17"/>
-      <c r="S6" s="17"/>
-      <c r="T6" s="17"/>
-      <c r="U6" s="17"/>
-      <c r="V6" s="17"/>
-      <c r="W6" s="17"/>
-      <c r="X6" s="17"/>
-      <c r="Y6" s="18"/>
-    </row>
-    <row r="7" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
@@ -1120,8 +904,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0671443-C51E-42ED-B6E9-3EA401076830}">
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDD70740-6FBF-43AF-83B0-7173CE1966F2}">
   <dimension ref="A1:Y8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1173,7 +957,7 @@
       <c r="L2" s="3"/>
       <c r="M2" s="4"/>
       <c r="N2" s="22" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="O2" s="23"/>
       <c r="P2" s="23"/>
@@ -1204,7 +988,496 @@
       <c r="L3" s="3"/>
       <c r="M3" s="4"/>
       <c r="N3" s="5" t="s">
-        <v>18</v>
+        <v>41</v>
+      </c>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="7"/>
+    </row>
+    <row r="4" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="6"/>
+      <c r="Y4" s="7"/>
+    </row>
+    <row r="5" spans="1:25" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="5">
+        <v>2.1</v>
+      </c>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+      <c r="Y5" s="12"/>
+    </row>
+    <row r="6" spans="1:25" ht="162" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
+      <c r="V6" s="17"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="17"/>
+      <c r="Y6" s="18"/>
+    </row>
+    <row r="7" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="5">
+        <v>6</v>
+      </c>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="7"/>
+    </row>
+    <row r="8" spans="1:25" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A7:M7"/>
+    <mergeCell ref="N7:Y7"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="N4:Y4"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="N5:Y5"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="N6:Y6"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="N1:Y1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="N2:Y2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="N3:Y3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Y8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:25" s="1" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+      <c r="T1" s="20"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="20"/>
+      <c r="X1" s="20"/>
+      <c r="Y1" s="21"/>
+    </row>
+    <row r="2" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="22">
+        <v>46043</v>
+      </c>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="7"/>
+    </row>
+    <row r="3" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="5">
+        <v>1</v>
+      </c>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="7"/>
+    </row>
+    <row r="4" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="6"/>
+      <c r="Y4" s="7"/>
+    </row>
+    <row r="5" spans="1:25" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+      <c r="X5" s="6"/>
+      <c r="Y5" s="7"/>
+    </row>
+    <row r="6" spans="1:25" ht="162" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
+      <c r="V6" s="17"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="17"/>
+      <c r="Y6" s="18"/>
+    </row>
+    <row r="7" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="5">
+        <v>1</v>
+      </c>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="7"/>
+    </row>
+    <row r="8" spans="1:25" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="N2:Y2"/>
+    <mergeCell ref="N3:Y3"/>
+    <mergeCell ref="N1:Y1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A7:M7"/>
+    <mergeCell ref="N4:Y4"/>
+    <mergeCell ref="N7:Y7"/>
+    <mergeCell ref="N6:Y6"/>
+    <mergeCell ref="N5:Y5"/>
+    <mergeCell ref="A5:M5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:Y8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:25" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+      <c r="T1" s="20"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="20"/>
+      <c r="X1" s="20"/>
+      <c r="Y1" s="21"/>
+    </row>
+    <row r="2" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="22">
+        <v>46055</v>
+      </c>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="24"/>
+    </row>
+    <row r="3" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="5">
+        <v>1</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
@@ -1265,8 +1538,8 @@
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
       <c r="M5" s="10"/>
-      <c r="N5" s="5" t="s">
-        <v>16</v>
+      <c r="N5" s="25" t="s">
+        <v>14</v>
       </c>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
@@ -1297,7 +1570,7 @@
       <c r="L6" s="14"/>
       <c r="M6" s="15"/>
       <c r="N6" s="16" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
@@ -1328,7 +1601,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="4"/>
       <c r="N7" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
@@ -1364,8 +1637,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBA59DE7-9D52-4D8D-BB67-DCC7DF70561E}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0671443-C51E-42ED-B6E9-3EA401076830}">
   <dimension ref="A1:Y8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1417,7 +1690,7 @@
       <c r="L2" s="3"/>
       <c r="M2" s="4"/>
       <c r="N2" s="22" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O2" s="23"/>
       <c r="P2" s="23"/>
@@ -1448,7 +1721,7 @@
       <c r="L3" s="3"/>
       <c r="M3" s="4"/>
       <c r="N3" s="5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
@@ -1510,7 +1783,7 @@
       <c r="L5" s="9"/>
       <c r="M5" s="10"/>
       <c r="N5" s="5" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
@@ -1541,7 +1814,7 @@
       <c r="L6" s="14"/>
       <c r="M6" s="15"/>
       <c r="N6" s="16" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
@@ -1572,7 +1845,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="4"/>
       <c r="N7" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
@@ -1608,8 +1881,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8E44654-2DBA-4543-9F3B-8D1F4B41F219}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBA59DE7-9D52-4D8D-BB67-DCC7DF70561E}">
   <dimension ref="A1:Y8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1661,7 +1934,7 @@
       <c r="L2" s="3"/>
       <c r="M2" s="4"/>
       <c r="N2" s="22" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="O2" s="23"/>
       <c r="P2" s="23"/>
@@ -1754,7 +2027,7 @@
       <c r="L5" s="9"/>
       <c r="M5" s="10"/>
       <c r="N5" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
@@ -1785,7 +2058,7 @@
       <c r="L6" s="14"/>
       <c r="M6" s="15"/>
       <c r="N6" s="16" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
@@ -1852,8 +2125,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9842BCB-B579-43DC-A36D-CBE39332E715}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8E44654-2DBA-4543-9F3B-8D1F4B41F219}">
   <dimension ref="A1:Y8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1904,8 +2177,8 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
       <c r="M2" s="4"/>
-      <c r="N2" s="22">
-        <v>46082</v>
+      <c r="N2" s="22" t="s">
+        <v>26</v>
       </c>
       <c r="O2" s="23"/>
       <c r="P2" s="23"/>
@@ -1935,8 +2208,8 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="4"/>
-      <c r="N3" s="5">
-        <v>1</v>
+      <c r="N3" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
@@ -1967,7 +2240,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="4"/>
       <c r="N4" s="5" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
@@ -1997,8 +2270,8 @@
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
       <c r="M5" s="10"/>
-      <c r="N5" s="5">
-        <v>2.1</v>
+      <c r="N5" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
@@ -2029,7 +2302,7 @@
       <c r="L6" s="14"/>
       <c r="M6" s="15"/>
       <c r="N6" s="16" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
@@ -2060,7 +2333,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="4"/>
       <c r="N7" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
@@ -2096,8 +2369,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A607B5F4-3455-4DA9-A7A8-A29D8063057C}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9842BCB-B579-43DC-A36D-CBE39332E715}">
   <dimension ref="A1:Y8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2148,8 +2421,8 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
       <c r="M2" s="4"/>
-      <c r="N2" s="22" t="s">
-        <v>29</v>
+      <c r="N2" s="22">
+        <v>46082</v>
       </c>
       <c r="O2" s="23"/>
       <c r="P2" s="23"/>
@@ -2179,8 +2452,8 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="4"/>
-      <c r="N3" s="5" t="s">
-        <v>21</v>
+      <c r="N3" s="5">
+        <v>1</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
@@ -2241,8 +2514,8 @@
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
       <c r="M5" s="10"/>
-      <c r="N5" s="5" t="s">
-        <v>30</v>
+      <c r="N5" s="5">
+        <v>2.1</v>
       </c>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
@@ -2273,7 +2546,7 @@
       <c r="L6" s="14"/>
       <c r="M6" s="15"/>
       <c r="N6" s="16" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
@@ -2304,7 +2577,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="4"/>
       <c r="N7" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
@@ -2340,8 +2613,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEA70D48-0F63-40A7-A614-2A774FBC305E}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A607B5F4-3455-4DA9-A7A8-A29D8063057C}">
   <dimension ref="A1:Y8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2393,7 +2666,7 @@
       <c r="L2" s="3"/>
       <c r="M2" s="4"/>
       <c r="N2" s="22" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="O2" s="23"/>
       <c r="P2" s="23"/>
@@ -2424,7 +2697,7 @@
       <c r="L3" s="3"/>
       <c r="M3" s="4"/>
       <c r="N3" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
@@ -2455,7 +2728,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="4"/>
       <c r="N4" s="5" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
@@ -2486,7 +2759,7 @@
       <c r="L5" s="9"/>
       <c r="M5" s="10"/>
       <c r="N5" s="5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
@@ -2517,7 +2790,7 @@
       <c r="L6" s="14"/>
       <c r="M6" s="15"/>
       <c r="N6" s="16" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
@@ -2548,7 +2821,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="4"/>
       <c r="N7" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
@@ -2582,4 +2855,248 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEA70D48-0F63-40A7-A614-2A774FBC305E}">
+  <dimension ref="A1:Y8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:25" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+      <c r="T1" s="20"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="20"/>
+      <c r="X1" s="20"/>
+      <c r="Y1" s="21"/>
+    </row>
+    <row r="2" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="24"/>
+    </row>
+    <row r="3" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="7"/>
+    </row>
+    <row r="4" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="6"/>
+      <c r="Y4" s="7"/>
+    </row>
+    <row r="5" spans="1:25" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+      <c r="Y5" s="12"/>
+    </row>
+    <row r="6" spans="1:25" ht="162" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
+      <c r="V6" s="17"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="17"/>
+      <c r="Y6" s="18"/>
+    </row>
+    <row r="7" spans="1:25" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="5">
+        <v>5</v>
+      </c>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="7"/>
+    </row>
+    <row r="8" spans="1:25" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="N1:Y1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="N2:Y2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="N3:Y3"/>
+    <mergeCell ref="A7:M7"/>
+    <mergeCell ref="N7:Y7"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="N4:Y4"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="N5:Y5"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="N6:Y6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>